<commit_message>
Subindo casos de teste
</commit_message>
<xml_diff>
--- a/documentação/Testes/Caso de Teste/UC06 - MANTER PACIENTES ASSOCIADOS.xlsx
+++ b/documentação/Testes/Caso de Teste/UC06 - MANTER PACIENTES ASSOCIADOS.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Casos de Teste" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Casos de Teste" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="78">
   <si>
     <t xml:space="preserve">Caso de Teste</t>
   </si>
@@ -64,13 +64,16 @@
     <t xml:space="preserve">-</t>
   </si>
   <si>
-    <t xml:space="preserve">Lista exibida com: foto (thumbnail), nome, idade, gênero, status e opções de edição</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lista carregada corretamente com todos os campos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OK</t>
+    <t xml:space="preserve">Lista exibida com: foto (thumbnail), nome, data de nascimento, sexo, status e opções de edição</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lista carregada corretamente com todos os campos exceto o campo de foto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOK</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> a thumbnail da foto não aparece corretamente</t>
   </si>
   <si>
     <t xml:space="preserve">CT02 - Cadastrar Novo Paciente (Sucesso)</t>
@@ -99,6 +102,9 @@
     <t xml:space="preserve">Paciente cadastrado com sucesso</t>
   </si>
   <si>
+    <t xml:space="preserve">OK</t>
+  </si>
+  <si>
     <t xml:space="preserve">CT03 - Cadastrar Paciente com CPF Inválido (FA1)</t>
   </si>
   <si>
@@ -180,7 +186,10 @@
     <t xml:space="preserve">Thumbnail é atualizado na lista</t>
   </si>
   <si>
-    <t xml:space="preserve">Foto atualizada corretamente</t>
+    <t xml:space="preserve">Foto atualizada corretamente porem thumbnail não carrega corretamente</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> foto atualiza porem thumbnail não aparece na lista</t>
   </si>
   <si>
     <t xml:space="preserve">CT07 - Tentar Enviar Foto Inválida (FA3)</t>
@@ -218,7 +227,10 @@
     <t xml:space="preserve">Status muda para "Inativo"; Paciente não aparece em agendamentos</t>
   </si>
   <si>
-    <t xml:space="preserve">Status alterado para "Inativo"</t>
+    <t xml:space="preserve">Não e possível desativar o paciente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ao clicar para desativar o paciente abre a aba para edição e não desativa o paciente</t>
   </si>
   <si>
     <t xml:space="preserve">CT09 - Reativar Paciente</t>
@@ -237,7 +249,7 @@
     <t xml:space="preserve">Status muda para "Ativo"; Paciente volta a aparecer em agendamentos</t>
   </si>
   <si>
-    <t xml:space="preserve">Status alterado para "Ativo"</t>
+    <t xml:space="preserve">Não é possível ativar o paciente</t>
   </si>
   <si>
     <t xml:space="preserve">CT10 - Validar Data de Nascimento Futura</t>
@@ -355,15 +367,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -379,12 +391,118 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultColWidth="32.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.04"/>
@@ -449,33 +567,33 @@
         <v>16</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>13</v>
@@ -483,28 +601,28 @@
     </row>
     <row r="4" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>16</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>13</v>
@@ -512,28 +630,28 @@
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>13</v>
@@ -541,28 +659,28 @@
     </row>
     <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>13</v>
@@ -570,147 +688,152 @@
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>16</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>13</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>16</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>13</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>16</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G15" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>